<commit_message>
results by template category
</commit_message>
<xml_diff>
--- a/data/templates.xlsx
+++ b/data/templates.xlsx
@@ -2124,7 +2124,7 @@
         <v>489</v>
       </c>
       <c r="C2" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="3" customHeight="1" ht="19.5">
@@ -2135,7 +2135,7 @@
         <v>490</v>
       </c>
       <c r="C3" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="4" customHeight="1" ht="19.5">
@@ -2146,7 +2146,7 @@
         <v>491</v>
       </c>
       <c r="C4" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="5" customHeight="1" ht="19.5">
@@ -2168,7 +2168,7 @@
         <v>493</v>
       </c>
       <c r="C6" s="7">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="7" customHeight="1" ht="19.5">
@@ -2179,7 +2179,7 @@
         <v>494</v>
       </c>
       <c r="C7" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="8" customHeight="1" ht="19.5">
@@ -2190,7 +2190,7 @@
         <v>495</v>
       </c>
       <c r="C8" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="9" customHeight="1" ht="19.5">
@@ -2201,7 +2201,7 @@
         <v>496</v>
       </c>
       <c r="C9" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="10" customHeight="1" ht="19.5">
@@ -2212,7 +2212,7 @@
         <v>497</v>
       </c>
       <c r="C10" s="7">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="11" customHeight="1" ht="19.5">
@@ -2223,7 +2223,7 @@
         <v>498</v>
       </c>
       <c r="C11" s="7">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row x14ac:dyDescent="0.25" r="12" customHeight="1" ht="19.5">
@@ -2234,7 +2234,7 @@
         <v>499</v>
       </c>
       <c r="C12" s="7">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>